<commit_message>
refactor: clean up project structure, fix 3 logic bugs, add DB scripts
- Fix movie2idx desync bug in engine_wrapper.py
- Fix cursor leak in public.py (trending/latest endpoints)
- Fix relative upload path bug in admin_movies.py (poster upload)
- Rename auth_refactored.py -> auth.py (remove legacy auth.py)
- Remove unused files: eda/ (root), model/ (root), main_eda.py,
  test_flow_stages.py, debug scripts, phase*_results.json
- Add .env.example for new machine setup
- Add scripts/dump_db.py and scripts/restore_db.py for DB portability
- Update .gitignore: track .pkl model files (now small ~4MB)
- Track output/models/*.pkl and uploads/posters/ for full deployment
</commit_message>
<xml_diff>
--- a/output/BaoCao_KiemThu_ToanDien.xlsx
+++ b/output/BaoCao_KiemThu_ToanDien.xlsx
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ngay thuc hien: 2026-05-19 16:36:55</t>
+          <t>Ngay thuc hien: 2026-06-06 19:11:30</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>{'total_movies': 3886, 'total_ratings': 1000245, 'total_users': 6044, 'real_users': 4, 'ts': 1779183210.5792756}</t>
+          <t>{'total_movies': 3986, 'total_ratings': 1001456, 'total_users': 6063, 'real_users': 13, 'rating_distribution': {'0.5': 30, '1.0': 56250, '1.5': 78, '2.0': 107647, '2.5': 80, '3.0': 261275, '3.5': 62, '4.0': 349138, '4.5': 331, '5.0': 226565}, 'top_rated_movies': [{'title': 'American Beauty (1999)', 'count': 3430}, {'title': 'Star Wars: Episode V - The Empire Strikes Back (1980)', 'count': 2993}, {'title': 'Star Wars: Episode IV - A New Hope (1977)', 'count': 2992}, {'title': 'Star Wars: Episode VI - Return of the Jedi (1983)', 'count': 2884}, {'title': 'Jurassic Park (1993)', 'count': 2672}], 'ts': 1780747718.0278013}</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>total_movies=3986</t>
+          <t>total_movies=4086</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>user_id=7020</t>
+          <t>user_id=7029</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>movie_ids=[4036, 3000, 4038, 4039, 4043, 4045, 4046]</t>
+          <t>movie_ids=[4136, 4137, 4138, 4139, 4143, 4145, 4146]</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>0/10 = 0% Animation</t>
+          <t>2/10 = 20% Animation</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>avg=3.27</t>
+          <t>avg=4.50</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>IDs: [6041, 6042, 6043, 6044, 6045, 6046, 6047, 6048, 6049, 6050]</t>
+          <t>IDs: [6051, 6052, 6053, 6054, 6055, 6056, 6057, 6058, 6059, 6060]</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Inserted 272 ratings</t>
+          <t>Inserted 308 ratings</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>target=275, actual=272</t>
+          <t>target=300, actual=308</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>before=1000253, after=1000525</t>
+          <t>before=1001464, after=1001772</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>before=1777542464, after=1779183357</t>
+          <t>before=1779210514, after=1780747876</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>User 6041: 20 recs via 'hybrid_foldin'</t>
+          <t>User 6051: 20 recs via 'hybrid_foldin'</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>User 6042: 20 recs via 'hybrid_foldin'</t>
+          <t>User 6052: 20 recs via 'hybrid_foldin'</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>User 6043: 20 recs via 'hybrid_foldin'</t>
+          <t>User 6053: 20 recs via 'hybrid_foldin'</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>User 6044: 20 recs via 'hybrid_foldin'</t>
+          <t>User 6054: 20 recs via 'hybrid_foldin'</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>User 6045: 20 recs via 'hybrid_foldin'</t>
+          <t>User 6055: 20 recs via 'hybrid_foldin'</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>User 6041: Diversity = 77.8%</t>
+          <t>User 6051: Diversity = 66.7%</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>14 unique genres in top-20</t>
+          <t>12 unique genres in top-20</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>User 6042: Diversity = 66.7%</t>
+          <t>User 6052: Diversity = 61.1%</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>12 unique genres in top-20</t>
+          <t>11 unique genres in top-20</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>User 6043: Diversity = 55.6%</t>
+          <t>User 6053: Diversity = 77.8%</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>10 unique genres in top-20</t>
+          <t>14 unique genres in top-20</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>User 6041: 0 new movies in top-20</t>
+          <t>User 6051: 0 new movies in top-20</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>User 6042: 0 new movies in top-20</t>
+          <t>User 6052: 0 new movies in top-20</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>User 6043: 0 new movies in top-20</t>
+          <t>User 6053: 0 new movies in top-20</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Users 6041 vs 6042: Jaccard=0.11</t>
+          <t>Users 6051 vs 6052: Jaccard=0.00</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>overlap=2/10, personalized=Yes</t>
+          <t>overlap=0/10, personalized=Yes</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Users 6041 vs 6043: Jaccard=0.00</t>
+          <t>Users 6051 vs 6053: Jaccard=0.11</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>overlap=0/10, personalized=Yes</t>
+          <t>overlap=2/10, personalized=Yes</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Users 6042 vs 6043: Jaccard=0.00</t>
+          <t>Users 6052 vs 6053: Jaccard=0.00</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>{"total_movies": 3986, "total_ratings": 1000525, "total_users": 6056, "real_users": 6, "ts": 1779183383.9167073}</t>
+          <t>{"total_movies": 4086, "total_ratings": 1001772, "total_users": 6075, "real_users": 15, "rating_distribution": {"0.5": 53, "1.0": 56276, "1.5": 105, "2.0": 107685, "2.5": 111, "3.0": 261304, "3.5": 89, "4.0": 349176, "4.5": 364, "5.0": 226609}, "top_rated_movies": [{"title": "American Beauty (1999)", "count": 3430}, {"title": "Star Wars: Episode V - The Empire Strikes Back (1980)", "count": 2993}, {"title": "Star Wars: Episode IV - A New Hope (1977)", "count": 2992}, {"title": "Star Wars: Episode VI - Return of the Jedi (1983)", "count": 2884}, {"title": "Jurassic Park (1993)", "count": 2672}], "ts": 1780747890.2754064}</t>
         </is>
       </c>
     </row>
@@ -2167,17 +2167,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1000253</t>
+          <t>1001464</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>1000525</t>
+          <t>1001772</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>+272</t>
+          <t>+308</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>3956</v>
+        <v>4056</v>
       </c>
       <c r="C2" s="17" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>3957</v>
+        <v>4057</v>
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>3958</v>
+        <v>4058</v>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>3959</v>
+        <v>4059</v>
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
@@ -2413,7 +2413,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>3960</v>
+        <v>4060</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>3961</v>
+        <v>4061</v>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
@@ -2449,7 +2449,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>3962</v>
+        <v>4062</v>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="14" t="n">
-        <v>3963</v>
+        <v>4063</v>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>3964</v>
+        <v>4064</v>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
@@ -2503,7 +2503,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="14" t="n">
-        <v>3965</v>
+        <v>4065</v>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="14" t="n">
-        <v>3966</v>
+        <v>4066</v>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>3967</v>
+        <v>4067</v>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>3968</v>
+        <v>4068</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
@@ -2575,7 +2575,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>3969</v>
+        <v>4069</v>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
@@ -2593,7 +2593,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>3970</v>
+        <v>4070</v>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>3971</v>
+        <v>4071</v>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
@@ -2629,7 +2629,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>3972</v>
+        <v>4072</v>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
@@ -2647,7 +2647,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="14" t="n">
-        <v>3973</v>
+        <v>4073</v>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="14" t="n">
-        <v>3974</v>
+        <v>4074</v>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
@@ -2683,7 +2683,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="14" t="n">
-        <v>3975</v>
+        <v>4075</v>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="14" t="n">
-        <v>3976</v>
+        <v>4076</v>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="14" t="n">
-        <v>3977</v>
+        <v>4077</v>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="14" t="n">
-        <v>3978</v>
+        <v>4078</v>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
@@ -2755,7 +2755,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="14" t="n">
-        <v>3979</v>
+        <v>4079</v>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="14" t="n">
-        <v>3980</v>
+        <v>4080</v>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
@@ -2791,7 +2791,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="14" t="n">
-        <v>3981</v>
+        <v>4081</v>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="14" t="n">
-        <v>3982</v>
+        <v>4082</v>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
@@ -2827,7 +2827,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="14" t="n">
-        <v>3983</v>
+        <v>4083</v>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
@@ -2845,7 +2845,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="14" t="n">
-        <v>3984</v>
+        <v>4084</v>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
@@ -2863,7 +2863,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="14" t="n">
-        <v>3985</v>
+        <v>4085</v>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
@@ -2881,7 +2881,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="14" t="n">
-        <v>3986</v>
+        <v>4086</v>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="14" t="n">
-        <v>3987</v>
+        <v>4087</v>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
@@ -2917,7 +2917,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="14" t="n">
-        <v>3988</v>
+        <v>4088</v>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="14" t="n">
-        <v>3989</v>
+        <v>4089</v>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
@@ -2953,7 +2953,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="14" t="n">
-        <v>3990</v>
+        <v>4090</v>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="14" t="n">
-        <v>3991</v>
+        <v>4091</v>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="14" t="n">
-        <v>3992</v>
+        <v>4092</v>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="14" t="n">
-        <v>3993</v>
+        <v>4093</v>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
@@ -3025,7 +3025,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="14" t="n">
-        <v>3994</v>
+        <v>4094</v>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="14" t="n">
-        <v>3995</v>
+        <v>4095</v>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
@@ -3061,7 +3061,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="14" t="n">
-        <v>3996</v>
+        <v>4096</v>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="14" t="n">
-        <v>3997</v>
+        <v>4097</v>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="14" t="n">
-        <v>3998</v>
+        <v>4098</v>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
@@ -3115,7 +3115,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="14" t="n">
-        <v>3999</v>
+        <v>4099</v>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="14" t="n">
-        <v>4000</v>
+        <v>4100</v>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="14" t="n">
-        <v>4001</v>
+        <v>4101</v>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="14" t="n">
-        <v>4002</v>
+        <v>4102</v>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
@@ -3187,7 +3187,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="14" t="n">
-        <v>4003</v>
+        <v>4103</v>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
@@ -3205,7 +3205,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="14" t="n">
-        <v>4004</v>
+        <v>4104</v>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="14" t="n">
-        <v>4005</v>
+        <v>4105</v>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="14" t="n">
-        <v>4006</v>
+        <v>4106</v>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
@@ -3259,7 +3259,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="14" t="n">
-        <v>4007</v>
+        <v>4107</v>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="14" t="n">
-        <v>4008</v>
+        <v>4108</v>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="14" t="n">
-        <v>4009</v>
+        <v>4109</v>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="14" t="n">
-        <v>4010</v>
+        <v>4110</v>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
@@ -3331,7 +3331,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="14" t="n">
-        <v>4011</v>
+        <v>4111</v>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
@@ -3349,7 +3349,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="14" t="n">
-        <v>4012</v>
+        <v>4112</v>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="14" t="n">
-        <v>4013</v>
+        <v>4113</v>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
@@ -3385,7 +3385,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="14" t="n">
-        <v>4014</v>
+        <v>4114</v>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
@@ -3403,7 +3403,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="14" t="n">
-        <v>4015</v>
+        <v>4115</v>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="14" t="n">
-        <v>4016</v>
+        <v>4116</v>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="14" t="n">
-        <v>4017</v>
+        <v>4117</v>
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="14" t="n">
-        <v>4018</v>
+        <v>4118</v>
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
@@ -3475,7 +3475,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="14" t="n">
-        <v>4019</v>
+        <v>4119</v>
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
@@ -3493,7 +3493,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="14" t="n">
-        <v>4020</v>
+        <v>4120</v>
       </c>
       <c r="C66" s="17" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="14" t="n">
-        <v>4021</v>
+        <v>4121</v>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
@@ -3529,7 +3529,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="14" t="n">
-        <v>4022</v>
+        <v>4122</v>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
@@ -3547,7 +3547,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="14" t="n">
-        <v>4023</v>
+        <v>4123</v>
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="14" t="n">
-        <v>4024</v>
+        <v>4124</v>
       </c>
       <c r="C70" s="17" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="14" t="n">
-        <v>4025</v>
+        <v>4125</v>
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="14" t="n">
-        <v>4026</v>
+        <v>4126</v>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
@@ -3619,7 +3619,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="14" t="n">
-        <v>4027</v>
+        <v>4127</v>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
@@ -3637,7 +3637,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="14" t="n">
-        <v>4028</v>
+        <v>4128</v>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
@@ -3655,7 +3655,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="14" t="n">
-        <v>4029</v>
+        <v>4129</v>
       </c>
       <c r="C75" s="17" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="14" t="n">
-        <v>4030</v>
+        <v>4130</v>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="14" t="n">
-        <v>4031</v>
+        <v>4131</v>
       </c>
       <c r="C77" s="17" t="inlineStr">
         <is>
@@ -3709,7 +3709,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="14" t="n">
-        <v>4032</v>
+        <v>4132</v>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="14" t="n">
-        <v>4033</v>
+        <v>4133</v>
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
@@ -3745,7 +3745,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="14" t="n">
-        <v>4034</v>
+        <v>4134</v>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
@@ -3763,7 +3763,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="14" t="n">
-        <v>4035</v>
+        <v>4135</v>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="14" t="n">
-        <v>4036</v>
+        <v>4136</v>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
@@ -3799,7 +3799,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="14" t="n">
-        <v>4037</v>
+        <v>4137</v>
       </c>
       <c r="C83" s="17" t="inlineStr">
         <is>
@@ -3817,7 +3817,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="14" t="n">
-        <v>4038</v>
+        <v>4138</v>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
@@ -3835,7 +3835,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="14" t="n">
-        <v>4039</v>
+        <v>4139</v>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="14" t="n">
-        <v>4040</v>
+        <v>4140</v>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
@@ -3871,7 +3871,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="14" t="n">
-        <v>4041</v>
+        <v>4141</v>
       </c>
       <c r="C87" s="17" t="inlineStr">
         <is>
@@ -3889,7 +3889,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="14" t="n">
-        <v>4042</v>
+        <v>4142</v>
       </c>
       <c r="C88" s="17" t="inlineStr">
         <is>
@@ -3907,7 +3907,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="14" t="n">
-        <v>4043</v>
+        <v>4143</v>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="14" t="n">
-        <v>4044</v>
+        <v>4144</v>
       </c>
       <c r="C90" s="17" t="inlineStr">
         <is>
@@ -3943,7 +3943,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="14" t="n">
-        <v>4045</v>
+        <v>4145</v>
       </c>
       <c r="C91" s="17" t="inlineStr">
         <is>
@@ -3961,7 +3961,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="14" t="n">
-        <v>4046</v>
+        <v>4146</v>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
@@ -3979,7 +3979,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="14" t="n">
-        <v>4047</v>
+        <v>4147</v>
       </c>
       <c r="C93" s="17" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="14" t="n">
-        <v>4048</v>
+        <v>4148</v>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
@@ -4015,7 +4015,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="14" t="n">
-        <v>4049</v>
+        <v>4149</v>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="14" t="n">
-        <v>4050</v>
+        <v>4150</v>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="14" t="n">
-        <v>4051</v>
+        <v>4151</v>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
@@ -4069,7 +4069,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="14" t="n">
-        <v>4052</v>
+        <v>4152</v>
       </c>
       <c r="C98" s="17" t="inlineStr">
         <is>
@@ -4087,7 +4087,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="14" t="n">
-        <v>4053</v>
+        <v>4153</v>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="14" t="n">
-        <v>4054</v>
+        <v>4154</v>
       </c>
       <c r="C100" s="17" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="14" t="n">
-        <v>4055</v>
+        <v>4155</v>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>

</xml_diff>